<commit_message>
pcb desing error -1,5h
</commit_message>
<xml_diff>
--- a/Hardware/PCB_Project/DIP_V01_Testing/PCB_Project/BOM_DIGIKEY_01_06_2026.xlsx
+++ b/Hardware/PCB_Project/DIP_V01_Testing/PCB_Project/BOM_DIGIKEY_01_06_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael Watzek\Documents\Diplom_Arbeit\Hardware\PCB_Project\DIP_V01_Testing\PCB_Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\Documents\Messung_von_Quanteneffecten_in_MOSFETs\Diplom_Arbeit\Hardware\PCB_Project\DIP_V01_Testing\PCB_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042B440C-0344-4732-A072-9D202E10F150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4306D1F8-B727-47BA-AB9B-0F4E8463E89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="712" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="712" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Muster" sheetId="8" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="94">
   <si>
     <t>HTL-Hollabrunn</t>
   </si>
@@ -153,33 +153,12 @@
     <t>digikey</t>
   </si>
   <si>
-    <t>100nF Capacitor Keramik 1206</t>
-  </si>
-  <si>
-    <t>4.7uF Capacitor Keramik 1206</t>
-  </si>
-  <si>
-    <t>1uF Capacitor Keramik 1206</t>
-  </si>
-  <si>
     <t>1N4148W-7 Diode SDO123_DIO</t>
   </si>
   <si>
     <t>BNC Elbow Connector</t>
   </si>
   <si>
-    <t>4.7k Resistor SMD 1206</t>
-  </si>
-  <si>
-    <t>3.9k Resistor SMD 1206</t>
-  </si>
-  <si>
-    <t>2.7k Resistor SMD 1206</t>
-  </si>
-  <si>
-    <t>Y0062100K000T9L Prezision 100k Resistor</t>
-  </si>
-  <si>
     <t>LT3042EMSE#TRPBF Ultralow Noise LDO 200mA</t>
   </si>
   <si>
@@ -195,9 +174,6 @@
     <t>TLV76733DGNR 1A 3,3V LDO</t>
   </si>
   <si>
-    <t>10uF Capacitor Keramik 1206 low ESR low ESL</t>
-  </si>
-  <si>
     <t>22pF Capacitor Keramik 1206 low ESR low ESL C0G/NP0</t>
   </si>
   <si>
@@ -249,12 +225,6 @@
     <t>https://www.digikey.at/de/products/detail/yageo/RT1206BRE0733KL/1080313</t>
   </si>
   <si>
-    <t>33k Resistor SMD 1206 0,1%</t>
-  </si>
-  <si>
-    <t>10k Resistor SMD 1206 0,1%</t>
-  </si>
-  <si>
     <t>P78.7KBCCT-ND</t>
   </si>
   <si>
@@ -306,12 +276,6 @@
     <t>https://www.digikey.at/de/products/detail/yageo/RT1206BRD0749K9L/1079848</t>
   </si>
   <si>
-    <t>Y0062-100KA-ND</t>
-  </si>
-  <si>
-    <t>https://www.digikey.at/de/products/detail/vpg-foil-resistors/Y0062100K000T9L/2609881?s=N4IgTCBcDaIJoAYEDYwEYkGkkICoE4AZEAXQF8g</t>
-  </si>
-  <si>
     <t>LT3042EMSE#TRPBFCT-ND</t>
   </si>
   <si>
@@ -367,6 +331,33 @@
   </si>
   <si>
     <t>49.9k Resistor SMD 1206 0,1% Dünnschicht</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 50V X7R 1206</t>
+  </si>
+  <si>
+    <t>CAP CER 10UF 16V X7R 1206 low ESL low ESR</t>
+  </si>
+  <si>
+    <t>CAP CER 4.7UF 50V X7R 1206</t>
+  </si>
+  <si>
+    <t>CAP CER 1UF 25V X7R 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 0.1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 33K OHM 0.1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 4.7K OHM 1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 3.9K OHM 1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 2.7K OHM 1% 1/4W 1206</t>
   </si>
 </sst>
 </file>
@@ -897,6 +888,27 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -906,6 +918,18 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -915,6 +939,54 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -928,11 +1000,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -968,85 +1038,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1355,7 +1346,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="15.6640625" customWidth="1"/>
@@ -1369,100 +1360,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="45" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="46"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="45" t="s">
+      <c r="B1" s="75"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="74" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="75"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="45" t="s">
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="47"/>
+      <c r="M1" s="76"/>
     </row>
     <row r="2" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="51" t="s">
+      <c r="B2" s="78"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="80" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="52"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="48" t="s">
+      <c r="E2" s="81"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="54">
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="83">
         <v>46174</v>
       </c>
-      <c r="M2" s="55"/>
+      <c r="M2" s="84"/>
     </row>
     <row r="3" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="45" t="s">
+      <c r="B3" s="75"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="46"/>
-      <c r="F3" s="45" t="s">
+      <c r="E3" s="75"/>
+      <c r="F3" s="74" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="47"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="47"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
+      <c r="J3" s="75"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="76"/>
     </row>
     <row r="4" spans="1:15" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="58"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="52"/>
       <c r="E4" s="8"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="63" t="s">
+      <c r="I4" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="64"/>
-      <c r="K4" s="62" t="s">
+      <c r="J4" s="58"/>
+      <c r="K4" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="L4" s="65"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="59"/>
-      <c r="B5" s="60"/>
-      <c r="C5" s="60"/>
-      <c r="D5" s="61"/>
+      <c r="A5" s="53"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="55"/>
       <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
@@ -1492,14 +1483,14 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="68"/>
+      <c r="A6" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="61"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="62"/>
       <c r="E6" s="24" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F6" s="11">
         <v>2</v>
@@ -1527,28 +1518,28 @@
         <v>0.93599999999999994</v>
       </c>
       <c r="M6" s="16">
-        <f t="shared" ref="M6:M29" si="0">L6</f>
+        <f t="shared" ref="M6:M28" si="0">L6</f>
         <v>0.93599999999999994</v>
       </c>
       <c r="O6" s="20" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="69" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="71"/>
+      <c r="A7" s="63" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="64"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="65"/>
       <c r="E7" s="24" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F7" s="17">
         <v>19</v>
       </c>
       <c r="G7" s="12">
-        <f t="shared" ref="G7:G29" si="1">F7</f>
+        <f t="shared" ref="G7:G28" si="1">F7</f>
         <v>19</v>
       </c>
       <c r="H7" s="13">
@@ -1574,18 +1565,18 @@
         <v>5.016</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="31"/>
+      <c r="A8" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="38"/>
       <c r="E8" s="24" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F8" s="18">
         <v>13</v>
@@ -1601,15 +1592,15 @@
         <v>0.27</v>
       </c>
       <c r="J8" s="23">
-        <f t="shared" ref="J8:J29" si="2">1.2*I8</f>
+        <f t="shared" ref="J8:J28" si="2">1.2*I8</f>
         <v>0.32400000000000001</v>
       </c>
       <c r="K8" s="14">
-        <f t="shared" ref="K8:K28" si="3">I8*H8*G8</f>
+        <f t="shared" ref="K8:K27" si="3">I8*H8*G8</f>
         <v>3.5100000000000002</v>
       </c>
       <c r="L8" s="15">
-        <f t="shared" ref="L8:L28" si="4">J8*H8*G8</f>
+        <f t="shared" ref="L8:L27" si="4">J8*H8*G8</f>
         <v>4.2119999999999997</v>
       </c>
       <c r="M8" s="16">
@@ -1617,18 +1608,18 @@
         <v>4.2119999999999997</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="31"/>
+      <c r="A9" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="38"/>
       <c r="E9" s="24" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="F9" s="17">
         <v>4</v>
@@ -1660,18 +1651,18 @@
         <v>1.6320000000000001</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="31"/>
+      <c r="A10" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="38"/>
       <c r="E10" s="24" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F10" s="19">
         <v>7</v>
@@ -1703,18 +1694,18 @@
         <v>1.5959999999999999</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="31"/>
+      <c r="A11" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="38"/>
       <c r="E11" s="24" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="F11" s="19">
         <v>4</v>
@@ -1746,18 +1737,18 @@
         <v>0.67200000000000004</v>
       </c>
       <c r="O11" s="20" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="31"/>
+      <c r="A12" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="38"/>
       <c r="E12" s="24" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F12" s="19">
         <v>4</v>
@@ -1789,18 +1780,18 @@
         <v>9.0239999999999991</v>
       </c>
       <c r="O12" s="20" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="31"/>
+      <c r="A13" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="38"/>
       <c r="E13" s="24" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F13" s="19">
         <v>10</v>
@@ -1832,18 +1823,18 @@
         <v>2.16</v>
       </c>
       <c r="O13" s="20" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31"/>
+      <c r="A14" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="38"/>
       <c r="E14" s="24" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F14" s="19">
         <v>1</v>
@@ -1875,18 +1866,18 @@
         <v>0.24</v>
       </c>
       <c r="O14" s="20" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="31"/>
+      <c r="A15" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38"/>
       <c r="E15" s="24" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F15" s="19">
         <v>2</v>
@@ -1918,18 +1909,18 @@
         <v>0.55200000000000005</v>
       </c>
       <c r="O15" s="20" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31"/>
+      <c r="A16" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="38"/>
       <c r="E16" s="24" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="F16" s="19">
         <v>3</v>
@@ -1961,18 +1952,18 @@
         <v>0.28800000000000003</v>
       </c>
       <c r="O16" s="20" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="31"/>
+      <c r="A17" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="38"/>
       <c r="E17" s="24" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="F17" s="19">
         <v>6</v>
@@ -2004,18 +1995,18 @@
         <v>0.57600000000000007</v>
       </c>
       <c r="O17" s="20" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="31"/>
+      <c r="A18" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="38"/>
       <c r="E18" s="24" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F18" s="19">
         <v>4</v>
@@ -2047,18 +2038,18 @@
         <v>0.38400000000000001</v>
       </c>
       <c r="O18" s="20" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
+      <c r="A19" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="38"/>
       <c r="E19" s="24" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F19" s="19">
         <v>2</v>
@@ -2090,18 +2081,18 @@
         <v>0.192</v>
       </c>
       <c r="O19" s="20" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
+      <c r="A20" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="38"/>
       <c r="E20" s="24" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F20" s="19">
         <v>1</v>
@@ -2133,18 +2124,18 @@
         <v>9.6000000000000002E-2</v>
       </c>
       <c r="O20" s="20" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="31"/>
+      <c r="A21" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38"/>
       <c r="E21" s="24" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="F21" s="19">
         <v>1</v>
@@ -2176,451 +2167,387 @@
         <v>0.216</v>
       </c>
       <c r="O21" s="20" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="31"/>
+      <c r="A22" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="38"/>
       <c r="E22" s="24" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="F22" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="12">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22" s="13">
         <v>1</v>
       </c>
       <c r="I22" s="21">
-        <v>31.74</v>
+        <v>6.43</v>
       </c>
       <c r="J22" s="23">
         <f t="shared" si="2"/>
-        <v>38.087999999999994</v>
+        <v>7.7159999999999993</v>
       </c>
       <c r="K22" s="14">
         <f t="shared" si="3"/>
-        <v>31.74</v>
+        <v>12.86</v>
       </c>
       <c r="L22" s="15">
         <f t="shared" si="4"/>
-        <v>38.087999999999994</v>
+        <v>15.431999999999999</v>
       </c>
       <c r="M22" s="16">
         <f t="shared" si="0"/>
-        <v>38.087999999999994</v>
+        <v>15.431999999999999</v>
       </c>
       <c r="O22" s="20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="31"/>
+      <c r="A23" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="38"/>
       <c r="E23" s="24" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="F23" s="19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="12">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23" s="13">
         <v>1</v>
       </c>
       <c r="I23" s="21">
-        <v>6.43</v>
+        <v>7.79</v>
       </c>
       <c r="J23" s="23">
         <f t="shared" si="2"/>
-        <v>7.7159999999999993</v>
+        <v>9.347999999999999</v>
       </c>
       <c r="K23" s="14">
         <f t="shared" si="3"/>
-        <v>12.86</v>
+        <v>7.79</v>
       </c>
       <c r="L23" s="15">
         <f t="shared" si="4"/>
-        <v>15.431999999999999</v>
+        <v>9.347999999999999</v>
       </c>
       <c r="M23" s="16">
         <f t="shared" si="0"/>
-        <v>15.431999999999999</v>
+        <v>9.347999999999999</v>
       </c>
       <c r="O23" s="20" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31"/>
+      <c r="A24" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="38"/>
       <c r="E24" s="24" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F24" s="19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G24" s="12">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H24" s="13">
         <v>1</v>
       </c>
       <c r="I24" s="21">
-        <v>7.79</v>
+        <v>1.5</v>
       </c>
       <c r="J24" s="23">
         <f t="shared" si="2"/>
-        <v>9.347999999999999</v>
+        <v>1.7999999999999998</v>
       </c>
       <c r="K24" s="14">
         <f t="shared" si="3"/>
-        <v>7.79</v>
+        <v>4.5</v>
       </c>
       <c r="L24" s="15">
         <f t="shared" si="4"/>
-        <v>9.347999999999999</v>
+        <v>5.3999999999999995</v>
       </c>
       <c r="M24" s="16">
         <f t="shared" si="0"/>
-        <v>9.347999999999999</v>
+        <v>5.3999999999999995</v>
       </c>
       <c r="O24" s="20" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="30"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="31"/>
+      <c r="A25" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="38"/>
       <c r="E25" s="24" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="F25" s="19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25" s="12">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H25" s="13">
         <v>1</v>
       </c>
       <c r="I25" s="21">
-        <v>1.5</v>
+        <v>0.82</v>
       </c>
       <c r="J25" s="23">
         <f t="shared" si="2"/>
-        <v>1.7999999999999998</v>
+        <v>0.98399999999999987</v>
       </c>
       <c r="K25" s="14">
         <f t="shared" si="3"/>
-        <v>4.5</v>
+        <v>0.82</v>
       </c>
       <c r="L25" s="15">
         <f t="shared" si="4"/>
-        <v>5.3999999999999995</v>
+        <v>0.98399999999999987</v>
       </c>
       <c r="M25" s="16">
         <f t="shared" si="0"/>
-        <v>5.3999999999999995</v>
+        <v>0.98399999999999987</v>
       </c>
       <c r="O25" s="20" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="B26" s="30"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="31"/>
+      <c r="A26" s="47" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="49"/>
       <c r="E26" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" s="19">
-        <v>1</v>
-      </c>
-      <c r="G26" s="12">
+        <v>80</v>
+      </c>
+      <c r="F26" s="18">
+        <v>2</v>
+      </c>
+      <c r="G26" s="25">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="H26" s="13">
-        <v>1</v>
-      </c>
-      <c r="I26" s="21">
-        <v>0.82</v>
-      </c>
-      <c r="J26" s="23">
+        <v>2</v>
+      </c>
+      <c r="H26" s="26">
+        <v>1</v>
+      </c>
+      <c r="I26" s="27">
+        <v>0.43</v>
+      </c>
+      <c r="J26" s="28">
         <f t="shared" si="2"/>
-        <v>0.98399999999999987</v>
+        <v>0.51600000000000001</v>
       </c>
       <c r="K26" s="14">
         <f t="shared" si="3"/>
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="L26" s="15">
         <f t="shared" si="4"/>
-        <v>0.98399999999999987</v>
+        <v>1.032</v>
       </c>
       <c r="M26" s="16">
         <f t="shared" si="0"/>
-        <v>0.98399999999999987</v>
+        <v>1.032</v>
       </c>
       <c r="O26" s="20" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="32" t="s">
-        <v>91</v>
-      </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="34"/>
+      <c r="A27" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="48"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="49"/>
       <c r="E27" s="24" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="F27" s="18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" s="25">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" s="26">
         <v>1</v>
       </c>
       <c r="I27" s="27">
-        <v>0.43</v>
+        <v>1.62</v>
       </c>
       <c r="J27" s="28">
         <f t="shared" si="2"/>
-        <v>0.51600000000000001</v>
+        <v>1.944</v>
       </c>
       <c r="K27" s="14">
         <f t="shared" si="3"/>
-        <v>0.86</v>
+        <v>1.62</v>
       </c>
       <c r="L27" s="15">
         <f t="shared" si="4"/>
-        <v>1.032</v>
+        <v>1.944</v>
       </c>
       <c r="M27" s="16">
         <f t="shared" si="0"/>
-        <v>1.032</v>
+        <v>1.944</v>
       </c>
       <c r="O27" s="20" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="34"/>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="38"/>
       <c r="E28" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="F28" s="18">
-        <v>1</v>
-      </c>
-      <c r="G28" s="25">
+        <v>73</v>
+      </c>
+      <c r="F28" s="19">
+        <v>1</v>
+      </c>
+      <c r="G28" s="12">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="H28" s="26">
-        <v>1</v>
-      </c>
-      <c r="I28" s="27">
-        <v>1.62</v>
-      </c>
-      <c r="J28" s="28">
+      <c r="H28" s="13">
+        <v>1</v>
+      </c>
+      <c r="I28" s="21">
+        <v>11.7</v>
+      </c>
+      <c r="J28" s="23">
         <f t="shared" si="2"/>
-        <v>1.944</v>
+        <v>14.04</v>
       </c>
       <c r="K28" s="14">
-        <f t="shared" si="3"/>
-        <v>1.62</v>
+        <f>I28*H28*G28</f>
+        <v>11.7</v>
       </c>
       <c r="L28" s="15">
-        <f t="shared" si="4"/>
-        <v>1.944</v>
+        <f>J28*H28*G28</f>
+        <v>14.04</v>
       </c>
       <c r="M28" s="16">
         <f t="shared" si="0"/>
-        <v>1.944</v>
+        <v>14.04</v>
       </c>
       <c r="O28" s="20" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="F29" s="19">
-        <v>1</v>
-      </c>
-      <c r="G29" s="12">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="H29" s="13">
-        <v>1</v>
-      </c>
-      <c r="I29" s="21">
-        <v>11.7</v>
-      </c>
-      <c r="J29" s="23">
-        <f t="shared" si="2"/>
-        <v>14.04</v>
-      </c>
-      <c r="K29" s="14">
-        <f>I29*H29*G29</f>
-        <v>11.7</v>
-      </c>
-      <c r="L29" s="15">
-        <f>J29*H29*G29</f>
-        <v>14.04</v>
-      </c>
-      <c r="M29" s="16">
-        <f t="shared" si="0"/>
-        <v>14.04</v>
-      </c>
-      <c r="O29" s="20" t="s">
-        <v>86</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="43"/>
+      <c r="I29" s="70" t="s">
+        <v>17</v>
+      </c>
+      <c r="J29" s="43"/>
+      <c r="K29" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="L29" s="40"/>
+      <c r="M29" s="29">
+        <f>SUM(M6:M28)</f>
+        <v>75.972000000000008</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="81" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="82"/>
-      <c r="C30" s="82"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="81" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="82"/>
-      <c r="G30" s="82"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="J30" s="40"/>
-      <c r="K30" s="79" t="s">
-        <v>18</v>
-      </c>
-      <c r="L30" s="80"/>
-      <c r="M30" s="72">
-        <f>SUM(M6:M29)</f>
-        <v>114.06</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="83"/>
-      <c r="B31" s="84"/>
-      <c r="C31" s="84"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="83"/>
-      <c r="F31" s="84"/>
-      <c r="G31" s="84"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="41"/>
-      <c r="J31" s="42"/>
-      <c r="K31" s="74" t="s">
+      <c r="A30" s="44"/>
+      <c r="B30" s="45"/>
+      <c r="C30" s="45"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="45"/>
+      <c r="G30" s="45"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="46"/>
+      <c r="K30" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="L31" s="75"/>
-      <c r="M31" s="73"/>
-    </row>
-    <row r="32" spans="1:15" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="76" t="s">
+      <c r="L30" s="32"/>
+      <c r="M30" s="30"/>
+    </row>
+    <row r="31" spans="1:15" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B32" s="77"/>
-      <c r="C32" s="77"/>
-      <c r="D32" s="78"/>
-      <c r="E32" s="76" t="s">
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="77"/>
-      <c r="G32" s="77"/>
-      <c r="H32" s="78"/>
-      <c r="I32" s="43"/>
-      <c r="J32" s="44"/>
-      <c r="K32" s="36"/>
-      <c r="L32" s="37"/>
-      <c r="M32" s="38"/>
-    </row>
-    <row r="36" spans="11:12" x14ac:dyDescent="0.3">
-      <c r="K36" s="35"/>
-      <c r="L36" s="35"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="72"/>
+      <c r="J31" s="73"/>
+      <c r="K31" s="67"/>
+      <c r="L31" s="68"/>
+      <c r="M31" s="69"/>
+    </row>
+    <row r="35" spans="11:12" x14ac:dyDescent="0.3">
+      <c r="K35" s="66"/>
+      <c r="L35" s="66"/>
     </row>
   </sheetData>
-  <mergeCells count="51">
-    <mergeCell ref="M30:M31"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="A30:D31"/>
-    <mergeCell ref="E30:H31"/>
-    <mergeCell ref="E32:H32"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A4:D5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="I31:J32"/>
+  <mergeCells count="50">
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J31"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="G1:K1"/>
@@ -2633,15 +2560,35 @@
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="F3:K3"/>
     <mergeCell ref="L3:M3"/>
+    <mergeCell ref="A4:D5"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A7:D7"/>
     <mergeCell ref="A20:D20"/>
+    <mergeCell ref="M29:M30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="A29:D30"/>
+    <mergeCell ref="E29:H30"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A24:D24"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O7" r:id="rId1" xr:uid="{ED586A59-BFEE-49BE-BB1E-047E5352E271}"/>
@@ -2658,18 +2605,17 @@
     <hyperlink ref="O19" r:id="rId12" xr:uid="{8AD09F14-6BD3-4674-B7A4-7966555F6D9C}"/>
     <hyperlink ref="O20" r:id="rId13" xr:uid="{0FA9C0DA-400B-4C54-83EE-1C1F289FFD37}"/>
     <hyperlink ref="O21" r:id="rId14" xr:uid="{F50CEB5F-75FA-47A0-A433-893F5323A4F2}"/>
-    <hyperlink ref="O22" r:id="rId15" xr:uid="{4EDF3955-2040-488A-AD97-A8361955C737}"/>
-    <hyperlink ref="O24" r:id="rId16" xr:uid="{5AAD0CB7-0B4D-451B-948B-CF520E287641}"/>
-    <hyperlink ref="O23" r:id="rId17" xr:uid="{4EC52342-A4F5-4940-990F-C16F68B6555F}"/>
-    <hyperlink ref="O25" r:id="rId18" xr:uid="{1BEF61F6-1485-47BD-B8DD-CB80D53A3A8E}"/>
-    <hyperlink ref="O26" r:id="rId19" xr:uid="{6B7F72A7-231D-4B29-BBC3-93EFAEAEAFE3}"/>
-    <hyperlink ref="O29" r:id="rId20" xr:uid="{C632BC62-DDCC-4722-8C0A-82BF835F3BAA}"/>
-    <hyperlink ref="O28" r:id="rId21" xr:uid="{2B0A17C3-A1E2-4E23-B0AF-AC882A73413D}"/>
-    <hyperlink ref="O27" r:id="rId22" xr:uid="{334C8E2F-0044-4D78-A4F7-3E0D1C8E663C}"/>
-    <hyperlink ref="O12" r:id="rId23" xr:uid="{A164AAD2-2EE5-4EF9-A42D-58E1C60E5339}"/>
+    <hyperlink ref="O23" r:id="rId15" xr:uid="{5AAD0CB7-0B4D-451B-948B-CF520E287641}"/>
+    <hyperlink ref="O22" r:id="rId16" xr:uid="{4EC52342-A4F5-4940-990F-C16F68B6555F}"/>
+    <hyperlink ref="O24" r:id="rId17" xr:uid="{1BEF61F6-1485-47BD-B8DD-CB80D53A3A8E}"/>
+    <hyperlink ref="O25" r:id="rId18" xr:uid="{6B7F72A7-231D-4B29-BBC3-93EFAEAEAFE3}"/>
+    <hyperlink ref="O28" r:id="rId19" xr:uid="{C632BC62-DDCC-4722-8C0A-82BF835F3BAA}"/>
+    <hyperlink ref="O27" r:id="rId20" xr:uid="{2B0A17C3-A1E2-4E23-B0AF-AC882A73413D}"/>
+    <hyperlink ref="O26" r:id="rId21" xr:uid="{334C8E2F-0044-4D78-A4F7-3E0D1C8E663C}"/>
+    <hyperlink ref="O12" r:id="rId22" xr:uid="{A164AAD2-2EE5-4EF9-A42D-58E1C60E5339}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="61" fitToWidth="0" orientation="landscape" r:id="rId24"/>
+  <pageSetup paperSize="9" scale="61" fitToWidth="0" orientation="landscape" r:id="rId23"/>
 </worksheet>
 </file>
 
@@ -2683,6 +2629,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101009657613A57DCA240BF1435E28856B226" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="5f3b321d472801a02a2afe67167e190e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3e560c01-df3e-4afb-8106-115af209489b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="42591c0612986ea9ea0f765279989779" ns2:_="">
     <xsd:import namespace="3e560c01-df3e-4afb-8106-115af209489b"/>
@@ -2820,12 +2772,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D205DF0-D259-4516-A145-B93EFE9EDE4A}">
   <ds:schemaRefs>
@@ -2835,6 +2781,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D3667C-8CCA-48C0-B4E3-78D1776152BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C81AFE02-87A2-490F-81E5-2F974BD2D586}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2850,13 +2805,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D3667C-8CCA-48C0-B4E3-78D1776152BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>